<commit_message>
fix node capa inputs and node capa const.
</commit_message>
<xml_diff>
--- a/03_rail_scheduling_dynamic_opt/opt_results_timetable_MON.xlsx
+++ b/03_rail_scheduling_dynamic_opt/opt_results_timetable_MON.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="28">
   <si>
     <t>Train</t>
   </si>
@@ -77,7 +77,7 @@
     <t>e6</t>
   </si>
   <si>
-    <t>e2</t>
+    <t>e4</t>
   </si>
   <si>
     <t>e7</t>
@@ -456,7 +456,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -566,25 +566,22 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E4">
+        <v>2</v>
+      </c>
+      <c r="F4" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="b">
         <v>1</v>
       </c>
-      <c r="F4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-      <c r="H4" t="b">
-        <v>0</v>
-      </c>
-      <c r="I4" t="b">
-        <v>0</v>
-      </c>
       <c r="J4" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:10">
@@ -592,63 +589,63 @@
         <v>11</v>
       </c>
       <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
         <v>15</v>
       </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
       <c r="E5">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G5">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H5" t="b">
         <v>0</v>
       </c>
       <c r="I5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F6" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G6">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
       </c>
       <c r="I6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7" spans="1:10">
@@ -656,30 +653,62 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
         <v>16</v>
       </c>
-      <c r="C7">
+      <c r="E7">
+        <v>2</v>
+      </c>
+      <c r="F7" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="b">
+        <v>0</v>
+      </c>
+      <c r="J7" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8">
         <v>3</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D8" t="s">
         <v>17</v>
       </c>
-      <c r="E7">
+      <c r="E8">
         <v>5</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F8" t="s">
         <v>23</v>
       </c>
-      <c r="G7">
-        <v>0</v>
-      </c>
-      <c r="H7" t="b">
-        <v>0</v>
-      </c>
-      <c r="I7" t="b">
-        <v>0</v>
-      </c>
-      <c r="J7" t="s">
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="b">
+        <v>0</v>
+      </c>
+      <c r="J8" t="s">
         <v>24</v>
       </c>
     </row>
@@ -734,7 +763,7 @@
         <v>15</v>
       </c>
       <c r="C4">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:3">
@@ -745,7 +774,7 @@
         <v>17</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="6" spans="1:3">

</xml_diff>

<commit_message>
add uk_real nodes_capacity data
</commit_message>
<xml_diff>
--- a/03_rail_scheduling_dynamic_opt/opt_results_timetable_MON.xlsx
+++ b/03_rail_scheduling_dynamic_opt/opt_results_timetable_MON.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="22">
   <si>
     <t>Train</t>
   </si>
@@ -62,12 +62,6 @@
     <t>n2</t>
   </si>
   <si>
-    <t>n3</t>
-  </si>
-  <si>
-    <t>n4</t>
-  </si>
-  <si>
     <t>n5</t>
   </si>
   <si>
@@ -77,19 +71,7 @@
     <t>e6</t>
   </si>
   <si>
-    <t>e4</t>
-  </si>
-  <si>
-    <t>e7</t>
-  </si>
-  <si>
-    <t>e3</t>
-  </si>
-  <si>
-    <t>e8</t>
-  </si>
-  <si>
-    <t>On-time &amp; complete</t>
+    <t>Delayed</t>
   </si>
   <si>
     <t>train</t>
@@ -456,7 +438,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:10">
@@ -508,19 +490,19 @@
         <v>2</v>
       </c>
       <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+      <c r="J2" t="s">
         <v>18</v>
-      </c>
-      <c r="G2">
-        <v>0</v>
-      </c>
-      <c r="H2" t="b">
-        <v>0</v>
-      </c>
-      <c r="I2" t="b">
-        <v>0</v>
-      </c>
-      <c r="J2" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:10">
@@ -531,19 +513,19 @@
         <v>14</v>
       </c>
       <c r="C3">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D3" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3">
+        <v>6</v>
+      </c>
+      <c r="F3" t="s">
         <v>17</v>
       </c>
-      <c r="E3">
-        <v>5</v>
-      </c>
-      <c r="F3" t="s">
-        <v>19</v>
-      </c>
       <c r="G3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="b">
         <v>0</v>
@@ -552,7 +534,7 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:10">
@@ -572,7 +554,7 @@
         <v>2</v>
       </c>
       <c r="F4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -592,16 +574,16 @@
         <v>14</v>
       </c>
       <c r="C5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" t="s">
         <v>15</v>
       </c>
       <c r="E5">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F5" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G5">
         <v>4</v>
@@ -618,25 +600,22 @@
     </row>
     <row r="6" spans="1:10">
       <c r="A6" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D6" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E6">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -653,19 +632,19 @@
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E7">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="G7">
         <v>0</v>
@@ -674,42 +653,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8">
-        <v>3</v>
-      </c>
-      <c r="D8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E8">
-        <v>5</v>
-      </c>
-      <c r="F8" t="s">
-        <v>23</v>
-      </c>
-      <c r="G8">
-        <v>0</v>
-      </c>
-      <c r="H8" t="b">
-        <v>0</v>
-      </c>
-      <c r="I8" t="b">
-        <v>0</v>
-      </c>
-      <c r="J8" t="s">
-        <v>24</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -719,18 +666,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="2" spans="1:3">
@@ -749,10 +696,10 @@
         <v>10</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C3">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -768,34 +715,12 @@
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C5">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>12</v>
-      </c>
-      <c r="B6" t="s">
-        <v>16</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3">
-      <c r="A7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B7" t="s">
-        <v>17</v>
-      </c>
-      <c r="C7">
         <v>0</v>
       </c>
     </row>

</xml_diff>